<commit_message>
Adjust sheet name for Excel constraints
Co-authored-by: mail135797 <mail135797@gmail.com>
</commit_message>
<xml_diff>
--- a/asin_variations.xlsx
+++ b/asin_variations.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="［SP］ ステビア - 商品 &gt; ［SP］ ラカンカ - 商品" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="・［SP］ ステビア - 商品&gt; ［SP］ ラカンカ - 商品" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +483,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>B0G9N4GV3K</t>
@@ -523,7 +522,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>B07QNVCL5Q</t>
@@ -541,7 +539,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>B0BTP4JK8N</t>
@@ -559,7 +556,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>B0BTP6P4XH</t>

</xml_diff>